<commit_message>
User Stories um Fotodefinition mit Winkeln erweitert
</commit_message>
<xml_diff>
--- a/Userstories.xlsx
+++ b/Userstories.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
   <si>
     <t xml:space="preserve">AGILE USER STORY TEMPLATE</t>
   </si>
@@ -52,6 +52,9 @@
     <t xml:space="preserve">STATUS</t>
   </si>
   <si>
+    <t xml:space="preserve">Anmerkung</t>
+  </si>
+  <si>
     <t xml:space="preserve">als Entwickler</t>
   </si>
   <si>
@@ -62,6 +65,19 @@
   </si>
   <si>
     <t xml:space="preserve">Bilder werden zyklisch auf SD Karte gespeichert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Als Entwickler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">den Machine-Learning-Algorithmus (im folgenden ML) mit Bilddaten versorgen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">den ML-Algorithmus anlernen kann</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pro aufgeführtem Winkel gibt es zwei Bilder auf zwei unterschiedlichen Hintergründen. Die Winkel geben den Aufnahmewinkel an, welcher von vorne gesehen um die horizontalachse des jeweiligen Schildes in Straßenrichtung (nach links also) verschoben ist. Das Auto soll dabei in normaler Fahrtrichtung zum Schild stehen.
+-10°, 0°, 10°, 25°, 35°, 45°, 55°, 60° (8 Winkel)</t>
   </si>
   <si>
     <t xml:space="preserve">An das Display soll ein Foto übertragen werden wenn auf dem Foto min. ein Schild erkannt wurde. Das erkannte Schild soll mit einem weißen Rahmen markiert werden.</t>
@@ -77,7 +93,7 @@
     <t xml:space="preserve">als Entwickler und Dozent</t>
   </si>
   <si>
-    <t xml:space="preserve">Ausgeben der Wahrscheinlichkeit dass das richtige Schild erkannt wurde</t>
+    <t xml:space="preserve">die Wahrscheinlichkeit, mit der das richtige Schild erkannt wurde ablesen können</t>
   </si>
   <si>
     <t xml:space="preserve">Damit ich einschätzen kann wie gut der ML-Code das Schild erkennt</t>
@@ -89,7 +105,7 @@
     <t xml:space="preserve">als Dozent</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich möchte ein Auto mit montierter Kamera haben</t>
+    <t xml:space="preserve">möchte ich ein Auto mit montierter Kamera haben</t>
   </si>
   <si>
     <t xml:space="preserve">Damit ich ein Simulationsfahrzeug habe</t>
@@ -108,6 +124,9 @@
   </si>
   <si>
     <t xml:space="preserve">Das Schild wird mit x% Wahrscheinlichkeit erkannt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erreichbare Wahrscheinlichkeit wird während dem Projektfortschritt ermittelt</t>
   </si>
   <si>
     <t xml:space="preserve">möchte ich ein Fahrerassistenzsystem auf ML-Basis, dass Schilder erkennen kann</t>
@@ -192,7 +211,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,6 +254,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -365,88 +390,100 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -534,9 +571,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1180800</xdr:colOff>
+      <xdr:colOff>1180440</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>285480</xdr:rowOff>
+      <xdr:rowOff>285120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -552,7 +589,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="368280" y="76320"/>
-          <a:ext cx="6491160" cy="780840"/>
+          <a:ext cx="6490800" cy="780480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -746,226 +783,312 @@
     <tabColor rgb="FF00B050"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B4:I18"/>
+  <dimension ref="B4:R19"/>
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="37.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="60.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="49.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="25.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="37.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="60.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="49.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="25.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="24.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="31.23"/>
   </cols>
   <sheetData>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" s="5" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="6" t="s">
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F7" s="5"/>
+      <c r="K7" s="0"/>
+      <c r="L7" s="0"/>
+      <c r="M7" s="0"/>
+      <c r="N7" s="0"/>
+      <c r="O7" s="0"/>
+      <c r="P7" s="0"/>
+      <c r="Q7" s="0"/>
+      <c r="R7" s="0"/>
+    </row>
+    <row r="8" s="6" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="9" t="s">
+      <c r="I8" s="10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" s="3" customFormat="true" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="10" t="n">
+      <c r="J8" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="K8" s="0"/>
+      <c r="L8" s="0"/>
+      <c r="M8" s="0"/>
+      <c r="N8" s="0"/>
+      <c r="O8" s="0"/>
+      <c r="P8" s="0"/>
+      <c r="Q8" s="0"/>
+      <c r="R8" s="0"/>
+    </row>
+    <row r="9" s="4" customFormat="true" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="11" t="s">
+      <c r="C9" s="12"/>
+      <c r="D9" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="E9" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="F9" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-    </row>
-    <row r="10" s="3" customFormat="true" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="10" t="n">
+      <c r="G9" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="0"/>
+      <c r="L9" s="0"/>
+      <c r="M9" s="0"/>
+      <c r="N9" s="0"/>
+      <c r="O9" s="0"/>
+      <c r="P9" s="0"/>
+      <c r="Q9" s="0"/>
+      <c r="R9" s="0"/>
+    </row>
+    <row r="10" s="4" customFormat="true" ht="100.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="12" t="s">
+      <c r="C10" s="12"/>
+      <c r="D10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="E10" s="13" t="s">
         <v>15</v>
       </c>
+      <c r="F10" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>17</v>
+      </c>
       <c r="H10" s="13"/>
-      <c r="I10" s="10"/>
-    </row>
-    <row r="11" s="3" customFormat="true" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="10" t="n">
+      <c r="I10" s="13"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="0"/>
+      <c r="L10" s="0"/>
+      <c r="M10" s="0"/>
+      <c r="N10" s="0"/>
+      <c r="O10" s="0"/>
+      <c r="P10" s="0"/>
+      <c r="Q10" s="0"/>
+      <c r="R10" s="0"/>
+    </row>
+    <row r="11" s="4" customFormat="true" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F11" s="10" t="s">
+      <c r="C11" s="12"/>
+      <c r="D11" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="F11" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="H11" s="13"/>
-      <c r="I11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="10" t="n">
+      <c r="G11" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="0"/>
+      <c r="L11" s="0"/>
+      <c r="M11" s="0"/>
+      <c r="N11" s="0"/>
+      <c r="O11" s="0"/>
+      <c r="P11" s="0"/>
+      <c r="Q11" s="0"/>
+      <c r="R11" s="0"/>
+    </row>
+    <row r="12" s="4" customFormat="true" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="10" t="s">
+      <c r="C12" s="12"/>
+      <c r="D12" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="E12" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="12" t="s">
+      <c r="F12" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="13"/>
+      <c r="G12" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="15"/>
       <c r="I12" s="15"/>
-    </row>
-    <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="10" t="n">
+      <c r="J12" s="12"/>
+      <c r="K12" s="0"/>
+      <c r="L12" s="0"/>
+      <c r="M12" s="0"/>
+      <c r="N12" s="0"/>
+      <c r="O12" s="0"/>
+      <c r="P12" s="0"/>
+      <c r="Q12" s="0"/>
+      <c r="R12" s="0"/>
+    </row>
+    <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" s="10" t="s">
+      <c r="C13" s="12"/>
+      <c r="D13" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="E13" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="G13" s="12" t="s">
+      <c r="F13" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="13"/>
-      <c r="I13" s="10"/>
+      <c r="G13" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="F14" s="10" t="s">
+      <c r="C14" s="12"/>
+      <c r="D14" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="E14" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="13"/>
-      <c r="I14" s="10"/>
+      <c r="F14" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="12" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
+      <c r="B15" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" s="12"/>
+      <c r="D15" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+    </row>
+    <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="B6:J6"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -987,39 +1110,39 @@
   <dimension ref="C4:D8"/>
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="37.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="19.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="37.42"/>
   </cols>
   <sheetData>
-    <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C4" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" s="13"/>
-    </row>
-    <row r="5" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C5" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="13"/>
-    </row>
-    <row r="6" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C6" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="13"/>
-    </row>
-    <row r="7" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C7" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="13"/>
-    </row>
-    <row r="8" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C8" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="13"/>
+    <row r="4" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C4" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="15"/>
+    </row>
+    <row r="5" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C5" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C6" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="15"/>
+    </row>
+    <row r="7" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C7" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="15"/>
+    </row>
+    <row r="8" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C8" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="15"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1041,53 +1164,53 @@
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="17" t="s">
-        <v>36</v>
+      <c r="B2" s="20" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="0" t="s">
-        <v>37</v>
+      <c r="B3" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="0" t="s">
-        <v>38</v>
+      <c r="B4" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="0" t="s">
-        <v>39</v>
+      <c r="B5" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="0" t="s">
-        <v>40</v>
+      <c r="B6" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="17" t="s">
-        <v>41</v>
+      <c r="B8" s="20" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="0" t="s">
-        <v>42</v>
+      <c r="B9" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0" t="s">
-        <v>43</v>
+      <c r="B10" s="1" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="0" t="s">
-        <v>44</v>
+      <c r="B11" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="0" t="s">
-        <v>45</v>
+      <c r="B12" s="1" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1110,43 +1233,43 @@
   <dimension ref="B2:B8"/>
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="68.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="68.29"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="18" t="s">
-        <v>46</v>
+      <c r="B2" s="21" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="19" t="s">
-        <v>47</v>
+      <c r="B3" s="22" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="19" t="s">
-        <v>48</v>
+      <c r="B4" s="22" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="19" t="s">
-        <v>49</v>
+      <c r="B5" s="22" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="19" t="s">
-        <v>50</v>
+      <c r="B6" s="22" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="19" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" s="3" customFormat="true" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="19" t="s">
-        <v>52</v>
+      <c r="B7" s="22" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" s="4" customFormat="true" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="22" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Userstory für Testdaten angepasst und das Diagramm über Trainingsdaten
</commit_message>
<xml_diff>
--- a/Userstories.xlsx
+++ b/Userstories.xlsx
@@ -76,8 +76,7 @@
     <t xml:space="preserve">den ML-Algorithmus anlernen kann</t>
   </si>
   <si>
-    <t xml:space="preserve">Pro aufgeführtem Winkel gibt es zwei Bilder auf zwei unterschiedlichen Hintergründen. Die Winkel geben den Aufnahmewinkel an, welcher von vorne gesehen um die horizontalachse des jeweiligen Schildes in Straßenrichtung (nach links also) verschoben ist. Das Auto soll dabei in normaler Fahrtrichtung zum Schild stehen.
--10°, 0°, 10°, 25°, 35°, 45°, 55°, 60° (8 Winkel)</t>
+    <t xml:space="preserve">Pro Schild gibt es mindestens 30 Bilder auf mindestens 3 verschiedenen Hintergründen. Das Auto wurde zwischen den Fotos langsam auf das Schild in normaler Fahrtrichtung zu bewegt.</t>
   </si>
   <si>
     <t xml:space="preserve">An das Display soll ein Foto übertragen werden wenn auf dem Foto min. ein Schild erkannt wurde. Das erkannte Schild soll mit einem weißen Rahmen markiert werden.</t>
@@ -211,7 +210,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -254,12 +253,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -390,11 +383,11 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -435,10 +428,6 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -471,19 +460,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -571,9 +560,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1180440</xdr:colOff>
+      <xdr:colOff>1180080</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>285120</xdr:rowOff>
+      <xdr:rowOff>284760</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -589,7 +578,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="368280" y="76320"/>
-          <a:ext cx="6490800" cy="780480"/>
+          <a:ext cx="6490440" cy="780120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -815,14 +804,14 @@
     </row>
     <row r="7" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F7" s="5"/>
-      <c r="K7" s="0"/>
-      <c r="L7" s="0"/>
-      <c r="M7" s="0"/>
-      <c r="N7" s="0"/>
-      <c r="O7" s="0"/>
-      <c r="P7" s="0"/>
-      <c r="Q7" s="0"/>
-      <c r="R7" s="0"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
     </row>
     <row r="8" s="6" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="7" t="s">
@@ -846,245 +835,245 @@
       <c r="H8" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J8" s="11" t="s">
+      <c r="J8" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="K8" s="0"/>
-      <c r="L8" s="0"/>
-      <c r="M8" s="0"/>
-      <c r="N8" s="0"/>
-      <c r="O8" s="0"/>
-      <c r="P8" s="0"/>
-      <c r="Q8" s="0"/>
-      <c r="R8" s="0"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
     </row>
     <row r="9" s="4" customFormat="true" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12" t="s">
+      <c r="C9" s="11"/>
+      <c r="D9" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="0"/>
-      <c r="L9" s="0"/>
-      <c r="M9" s="0"/>
-      <c r="N9" s="0"/>
-      <c r="O9" s="0"/>
-      <c r="P9" s="0"/>
-      <c r="Q9" s="0"/>
-      <c r="R9" s="0"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
+      <c r="R9" s="1"/>
     </row>
     <row r="10" s="4" customFormat="true" ht="100.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12" t="s">
+      <c r="C10" s="11"/>
+      <c r="D10" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="0"/>
-      <c r="L10" s="0"/>
-      <c r="M10" s="0"/>
-      <c r="N10" s="0"/>
-      <c r="O10" s="0"/>
-      <c r="P10" s="0"/>
-      <c r="Q10" s="0"/>
-      <c r="R10" s="0"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+      <c r="R10" s="1"/>
     </row>
     <row r="11" s="4" customFormat="true" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12" t="s">
+      <c r="C11" s="11"/>
+      <c r="D11" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="0"/>
-      <c r="L11" s="0"/>
-      <c r="M11" s="0"/>
-      <c r="N11" s="0"/>
-      <c r="O11" s="0"/>
-      <c r="P11" s="0"/>
-      <c r="Q11" s="0"/>
-      <c r="R11" s="0"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1"/>
+      <c r="R11" s="1"/>
     </row>
     <row r="12" s="4" customFormat="true" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12" t="s">
+      <c r="C12" s="11"/>
+      <c r="D12" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="G12" s="14" t="s">
+      <c r="G12" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="0"/>
-      <c r="L12" s="0"/>
-      <c r="M12" s="0"/>
-      <c r="N12" s="0"/>
-      <c r="O12" s="0"/>
-      <c r="P12" s="0"/>
-      <c r="Q12" s="0"/>
-      <c r="R12" s="0"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="1"/>
+      <c r="Q12" s="1"/>
+      <c r="R12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="17" t="s">
+      <c r="C13" s="11"/>
+      <c r="D13" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="F13" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="G13" s="14" t="s">
+      <c r="G13" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="18"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="17"/>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12" t="s">
+      <c r="C14" s="11"/>
+      <c r="D14" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="G14" s="14" t="s">
+      <c r="G14" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="12" t="s">
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="11" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="17" t="s">
+      <c r="C15" s="11"/>
+      <c r="D15" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="G15" s="14" t="s">
+      <c r="G15" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="12"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1115,34 +1104,34 @@
   </cols>
   <sheetData>
     <row r="4" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="15"/>
+      <c r="D4" s="14"/>
     </row>
     <row r="5" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="15"/>
+      <c r="D5" s="14"/>
     </row>
     <row r="6" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="15"/>
+      <c r="D6" s="14"/>
     </row>
     <row r="7" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="15"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="15"/>
+      <c r="D8" s="14"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1164,7 +1153,7 @@
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="19" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1189,7 +1178,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="19" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1238,37 +1227,37 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="21" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="21" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="8" s="4" customFormat="true" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="21" t="s">
         <v>58</v>
       </c>
     </row>

</xml_diff>

<commit_message>
User-Story 2 Akzeptanzkriterium erfüllt
</commit_message>
<xml_diff>
--- a/Userstories.xlsx
+++ b/Userstories.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
   <si>
     <t xml:space="preserve">AGILE USER STORY TEMPLATE</t>
   </si>
@@ -64,7 +64,13 @@
     <t xml:space="preserve">Damit ich Bildmaterial für meinen Algorithmus habe</t>
   </si>
   <si>
-    <t xml:space="preserve">Bilder werden zyklisch auf SD Karte gespeichert</t>
+    <t xml:space="preserve">Bilder können auf SD Karte gespeichert werden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Akzeptanzkriterium erfüllt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siehe Hilfsanwendung Fotoapparat</t>
   </si>
   <si>
     <t xml:space="preserve">Als Entwickler</t>
@@ -210,7 +216,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -253,6 +259,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -383,11 +395,11 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -440,6 +452,10 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -460,19 +476,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -560,9 +576,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1180080</xdr:colOff>
+      <xdr:colOff>1179720</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>284760</xdr:rowOff>
+      <xdr:rowOff>284400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -578,7 +594,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="368280" y="76320"/>
-          <a:ext cx="6490440" cy="780120"/>
+          <a:ext cx="6490080" cy="779760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -868,8 +884,12 @@
         <v>13</v>
       </c>
       <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
+      <c r="I9" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
@@ -885,19 +905,21 @@
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
       <c r="J10" s="12"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -916,17 +938,17 @@
       <c r="D11" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
+      <c r="F11" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
       <c r="J11" s="11"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
@@ -943,19 +965,19 @@
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>24</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
+        <v>25</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
       <c r="J12" s="11"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
@@ -971,21 +993,21 @@
         <v>5</v>
       </c>
       <c r="C13" s="11"/>
-      <c r="D13" s="16" t="s">
-        <v>25</v>
+      <c r="D13" s="17" t="s">
+        <v>27</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="17"/>
+        <v>29</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="11" t="n">
@@ -993,21 +1015,21 @@
       </c>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="G14" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
+        <v>33</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
       <c r="J14" s="11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1015,20 +1037,20 @@
         <v>7</v>
       </c>
       <c r="C15" s="11"/>
-      <c r="D15" s="16" t="s">
-        <v>25</v>
+      <c r="D15" s="17" t="s">
+        <v>27</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="G15" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
+        <v>37</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
       <c r="J15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1104,34 +1126,34 @@
   </cols>
   <sheetData>
     <row r="4" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C4" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="14"/>
+      <c r="C4" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C5" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="14"/>
+      <c r="C5" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C6" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D6" s="14"/>
+      <c r="C6" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="15"/>
     </row>
     <row r="7" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C7" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="14"/>
+      <c r="C7" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="15"/>
     </row>
     <row r="8" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C8" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="14"/>
+      <c r="C8" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="15"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1153,53 +1175,53 @@
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="19" t="s">
-        <v>42</v>
+      <c r="B2" s="20" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="19" t="s">
-        <v>47</v>
+      <c r="B8" s="20" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1227,38 +1249,38 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="20" t="s">
-        <v>52</v>
+      <c r="B2" s="21" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="21" t="s">
-        <v>53</v>
+      <c r="B3" s="22" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="21" t="s">
-        <v>54</v>
+      <c r="B4" s="22" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="21" t="s">
-        <v>55</v>
+      <c r="B5" s="22" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="21" t="s">
-        <v>56</v>
+      <c r="B6" s="22" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="21" t="s">
-        <v>57</v>
+      <c r="B7" s="22" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="8" s="4" customFormat="true" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="21" t="s">
-        <v>58</v>
+      <c r="B8" s="22" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Projektdokumentation mit Meetingänderungen aktualisiert
</commit_message>
<xml_diff>
--- a/Userstories.xlsx
+++ b/Userstories.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="64">
   <si>
     <t xml:space="preserve">AGILE USER STORY TEMPLATE</t>
   </si>
@@ -95,6 +95,10 @@
 Um alle als Schild erkannte Bereiche wird ein weißer Rahmen gelegt.</t>
   </si>
   <si>
+    <t xml:space="preserve">Wurde aus Zeitmangel
+Nicht umgesetzt</t>
+  </si>
+  <si>
     <t xml:space="preserve">als Entwickler und Dozent</t>
   </si>
   <si>
@@ -119,6 +123,9 @@
     <t xml:space="preserve">Kameramodul auf Legofahrzeug befestigt. Legofahrzeug kann verschoben werden ohne, dass das Modul herunterfallen kann. </t>
   </si>
   <si>
+    <t xml:space="preserve">Gehäuse für Board inklusive BlueBrixx Befestigung ist angefertigt</t>
+  </si>
+  <si>
     <t xml:space="preserve">als Lego-Autofahrer</t>
   </si>
   <si>
@@ -129,6 +136,11 @@
   </si>
   <si>
     <t xml:space="preserve">Das Schild wird mit x% Wahrscheinlichkeit erkannt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Akzeptanzkriterium erfüllt
+MATLAB erreicht 99% bei den Validierungsdaten
+Für OpenMV gibt es noch keinen Messwert</t>
   </si>
   <si>
     <t xml:space="preserve">Erreichbare Wahrscheinlichkeit wird während dem Projektfortschritt ermittelt</t>
@@ -452,10 +464,6 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -468,11 +476,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -576,9 +588,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1179720</xdr:colOff>
+      <xdr:colOff>1179360</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>284400</xdr:rowOff>
+      <xdr:rowOff>284040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -594,7 +606,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="368280" y="76320"/>
-          <a:ext cx="6490080" cy="779760"/>
+          <a:ext cx="6489720" cy="779400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -799,7 +811,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="60.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="49.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="25.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="24.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="41.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="31.23"/>
   </cols>
   <sheetData>
@@ -884,7 +896,7 @@
         <v>13</v>
       </c>
       <c r="H9" s="12"/>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="12" t="s">
         <v>14</v>
       </c>
       <c r="J9" s="12" t="s">
@@ -930,7 +942,7 @@
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
     </row>
-    <row r="11" s="4" customFormat="true" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" s="4" customFormat="true" ht="52.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="11" t="n">
         <v>3</v>
       </c>
@@ -938,17 +950,19 @@
       <c r="D11" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="13" t="s">
+        <v>23</v>
+      </c>
       <c r="J11" s="11"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
@@ -965,19 +979,21 @@
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="14"/>
+      <c r="I12" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
       <c r="J12" s="11"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
@@ -994,20 +1010,24 @@
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G13" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="18"/>
+      <c r="G13" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J13" s="18" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="11" t="n">
@@ -1015,21 +1035,23 @@
       </c>
       <c r="C14" s="11"/>
       <c r="D14" s="11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
+        <v>35</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14" s="14"/>
+      <c r="I14" s="13" t="s">
+        <v>37</v>
+      </c>
       <c r="J14" s="11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1038,19 +1060,21 @@
       </c>
       <c r="C15" s="11"/>
       <c r="D15" s="17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="G15" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
+        <v>40</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14" t="s">
+        <v>14</v>
+      </c>
       <c r="J15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1127,33 +1151,33 @@
   <sheetData>
     <row r="4" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C4" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="15"/>
+        <v>42</v>
+      </c>
+      <c r="D4" s="14"/>
     </row>
     <row r="5" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C5" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="D5" s="15"/>
+        <v>43</v>
+      </c>
+      <c r="D5" s="14"/>
     </row>
     <row r="6" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C6" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" s="15"/>
+        <v>44</v>
+      </c>
+      <c r="D6" s="14"/>
     </row>
     <row r="7" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C7" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" s="15"/>
+        <v>45</v>
+      </c>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" s="4" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C8" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="D8" s="15"/>
+        <v>46</v>
+      </c>
+      <c r="D8" s="14"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1176,52 +1200,52 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="20" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="20" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1250,37 +1274,37 @@
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="22" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="22" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="22" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="22" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="22" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" s="4" customFormat="true" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="22" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>